<commit_message>
AMS FREEZONE: Final Enterprise ERP Beast-Mode (v12)
- Hybrid AI-Wizard Engine: AI OCR pre-fills the Wizard for a zero-manual-entry flow.
- Premium Dark Theme: Redesigned all dialogs and Wizards with corporate dark styling.
- Legendary GL: Integrated Accounting with P&L, COA, and Trial Balance.
- Dashboard v12: Actionable critical lists and profit analytics.
- Pro Max++ Docs: Enlarged logo, corporate branding, and internal/external PDF viewing.
- Resilient Searching: Integrated QCompleter for fluid item selection.
- Global Date Tools: Single-click Batch Date overrides for inbound movements.
- Unshakable Stability: Re-engineered layout disposal and thread-safe DB pooling.
- Scale Ready: 100+ record templates and massive enterprise seeding.

Co-authored-by: cisentinel01-collab <282014271+cisentinel01-collab@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/example/items_large_template.xlsx
+++ b/example/items_large_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F101"/>
+  <dimension ref="A1:H101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -447,21 +447,31 @@
           <t>Current Stock</t>
         </is>
       </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>Production Date</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>Expiry Date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>SKU-BATCH-001</t>
+          <t>SKU-ERP-0001</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 1</t>
+          <t>Enterprise High-Grade Part 1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -470,26 +480,36 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="F2" t="n">
-        <v>343</v>
+        <v>207</v>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>SKU-BATCH-002</t>
+          <t>SKU-ERP-0002</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 2</t>
+          <t>Enterprise High-Grade Part 2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -498,26 +518,36 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
       <c r="F3" t="n">
-        <v>355</v>
+        <v>70</v>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>SKU-BATCH-003</t>
+          <t>SKU-ERP-0003</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 3</t>
+          <t>Enterprise High-Grade Part 3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -526,26 +556,36 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>46</v>
+        <v>18</v>
       </c>
       <c r="F4" t="n">
-        <v>63</v>
+        <v>633</v>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>SKU-BATCH-004</t>
+          <t>SKU-ERP-0004</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 4</t>
+          <t>Enterprise High-Grade Part 4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -554,21 +594,31 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="F5" t="n">
-        <v>367</v>
+        <v>412</v>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>SKU-BATCH-005</t>
+          <t>SKU-ERP-0005</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 5</t>
+          <t>Enterprise High-Grade Part 5</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -582,26 +632,36 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F6" t="n">
-        <v>50</v>
+        <v>151</v>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>SKU-BATCH-006</t>
+          <t>SKU-ERP-0006</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 6</t>
+          <t>Enterprise High-Grade Part 6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -610,26 +670,36 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="F7" t="n">
-        <v>131</v>
+        <v>452</v>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>SKU-BATCH-007</t>
+          <t>SKU-ERP-0007</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 7</t>
+          <t>Enterprise High-Grade Part 7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -638,26 +708,36 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F8" t="n">
-        <v>445</v>
+        <v>731</v>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>SKU-BATCH-008</t>
+          <t>SKU-ERP-0008</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 8</t>
+          <t>Enterprise High-Grade Part 8</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -666,26 +746,36 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>41</v>
+        <v>25</v>
       </c>
       <c r="F9" t="n">
-        <v>454</v>
+        <v>251</v>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>SKU-BATCH-009</t>
+          <t>SKU-ERP-0009</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 9</t>
+          <t>Enterprise High-Grade Part 9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -694,26 +784,36 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="F10" t="n">
-        <v>336</v>
+        <v>668</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>SKU-BATCH-010</t>
+          <t>SKU-ERP-0010</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 10</t>
+          <t>Enterprise High-Grade Part 10</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -722,26 +822,36 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>50</v>
+        <v>43</v>
       </c>
       <c r="F11" t="n">
-        <v>481</v>
+        <v>199</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>SKU-BATCH-011</t>
+          <t>SKU-ERP-0011</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 11</t>
+          <t>Enterprise High-Grade Part 11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -750,26 +860,36 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="F12" t="n">
-        <v>264</v>
+        <v>990</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>SKU-BATCH-012</t>
+          <t>SKU-ERP-0012</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 12</t>
+          <t>Enterprise High-Grade Part 12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -778,26 +898,36 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="F13" t="n">
-        <v>214</v>
+        <v>157</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>SKU-BATCH-013</t>
+          <t>SKU-ERP-0013</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 13</t>
+          <t>Enterprise High-Grade Part 13</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -806,21 +936,31 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>16</v>
+        <v>41</v>
       </c>
       <c r="F14" t="n">
-        <v>467</v>
+        <v>474</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SKU-BATCH-014</t>
+          <t>SKU-ERP-0014</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 14</t>
+          <t>Enterprise High-Grade Part 14</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -834,26 +974,36 @@
         </is>
       </c>
       <c r="E15" t="n">
-        <v>26</v>
+        <v>31</v>
       </c>
       <c r="F15" t="n">
-        <v>126</v>
+        <v>202</v>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SKU-BATCH-015</t>
+          <t>SKU-ERP-0015</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 15</t>
+          <t>Enterprise High-Grade Part 15</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -862,26 +1012,36 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F16" t="n">
-        <v>312</v>
+        <v>893</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>SKU-BATCH-016</t>
+          <t>SKU-ERP-0016</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 16</t>
+          <t>Enterprise High-Grade Part 16</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -890,26 +1050,36 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>41</v>
+        <v>48</v>
       </c>
       <c r="F17" t="n">
-        <v>371</v>
+        <v>836</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>SKU-BATCH-017</t>
+          <t>SKU-ERP-0017</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 17</t>
+          <t>Enterprise High-Grade Part 17</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -918,21 +1088,31 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>23</v>
+        <v>41</v>
       </c>
       <c r="F18" t="n">
-        <v>66</v>
+        <v>85</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>SKU-BATCH-018</t>
+          <t>SKU-ERP-0018</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 18</t>
+          <t>Enterprise High-Grade Part 18</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -946,26 +1126,36 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="F19" t="n">
-        <v>216</v>
+        <v>105</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>SKU-BATCH-019</t>
+          <t>SKU-ERP-0019</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 19</t>
+          <t>Enterprise High-Grade Part 19</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -974,21 +1164,31 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="F20" t="n">
-        <v>175</v>
+        <v>97</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>SKU-BATCH-020</t>
+          <t>SKU-ERP-0020</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 20</t>
+          <t>Enterprise High-Grade Part 20</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1002,21 +1202,31 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>28</v>
+        <v>47</v>
       </c>
       <c r="F21" t="n">
-        <v>348</v>
+        <v>534</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>SKU-BATCH-021</t>
+          <t>SKU-ERP-0021</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 21</t>
+          <t>Enterprise High-Grade Part 21</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -1030,26 +1240,36 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>47</v>
+        <v>37</v>
       </c>
       <c r="F22" t="n">
-        <v>52</v>
+        <v>726</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>SKU-BATCH-022</t>
+          <t>SKU-ERP-0022</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 22</t>
+          <t>Enterprise High-Grade Part 22</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -1058,21 +1278,31 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>37</v>
+        <v>29</v>
       </c>
       <c r="F23" t="n">
-        <v>359</v>
+        <v>377</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>SKU-BATCH-023</t>
+          <t>SKU-ERP-0023</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 23</t>
+          <t>Enterprise High-Grade Part 23</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -1086,26 +1316,36 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="F24" t="n">
-        <v>114</v>
+        <v>536</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SKU-BATCH-024</t>
+          <t>SKU-ERP-0024</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 24</t>
+          <t>Enterprise High-Grade Part 24</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -1114,26 +1354,36 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="F25" t="n">
-        <v>145</v>
+        <v>113</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>SKU-BATCH-025</t>
+          <t>SKU-ERP-0025</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 25</t>
+          <t>Enterprise High-Grade Part 25</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -1142,26 +1392,36 @@
         </is>
       </c>
       <c r="E26" t="n">
-        <v>42</v>
+        <v>36</v>
       </c>
       <c r="F26" t="n">
-        <v>291</v>
+        <v>578</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>SKU-BATCH-026</t>
+          <t>SKU-ERP-0026</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 26</t>
+          <t>Enterprise High-Grade Part 26</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -1170,26 +1430,36 @@
         </is>
       </c>
       <c r="E27" t="n">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="F27" t="n">
-        <v>79</v>
+        <v>511</v>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SKU-BATCH-027</t>
+          <t>SKU-ERP-0027</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 27</t>
+          <t>Enterprise High-Grade Part 27</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -1198,26 +1468,36 @@
         </is>
       </c>
       <c r="E28" t="n">
-        <v>45</v>
+        <v>26</v>
       </c>
       <c r="F28" t="n">
-        <v>310</v>
+        <v>764</v>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SKU-BATCH-028</t>
+          <t>SKU-ERP-0028</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 28</t>
+          <t>Enterprise High-Grade Part 28</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -1226,26 +1506,36 @@
         </is>
       </c>
       <c r="E29" t="n">
-        <v>45</v>
+        <v>35</v>
       </c>
       <c r="F29" t="n">
-        <v>289</v>
+        <v>91</v>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>SKU-BATCH-029</t>
+          <t>SKU-ERP-0029</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 29</t>
+          <t>Enterprise High-Grade Part 29</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -1254,26 +1544,36 @@
         </is>
       </c>
       <c r="E30" t="n">
-        <v>33</v>
+        <v>39</v>
       </c>
       <c r="F30" t="n">
-        <v>74</v>
+        <v>705</v>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>SKU-BATCH-030</t>
+          <t>SKU-ERP-0030</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 30</t>
+          <t>Enterprise High-Grade Part 30</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -1282,21 +1582,31 @@
         </is>
       </c>
       <c r="E31" t="n">
-        <v>16</v>
+        <v>32</v>
       </c>
       <c r="F31" t="n">
-        <v>478</v>
+        <v>670</v>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SKU-BATCH-031</t>
+          <t>SKU-ERP-0031</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 31</t>
+          <t>Enterprise High-Grade Part 31</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1310,26 +1620,36 @@
         </is>
       </c>
       <c r="E32" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="F32" t="n">
-        <v>314</v>
+        <v>994</v>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SKU-BATCH-032</t>
+          <t>SKU-ERP-0032</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 32</t>
+          <t>Enterprise High-Grade Part 32</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -1338,21 +1658,31 @@
         </is>
       </c>
       <c r="E33" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F33" t="n">
-        <v>357</v>
+        <v>257</v>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SKU-BATCH-033</t>
+          <t>SKU-ERP-0033</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 33</t>
+          <t>Enterprise High-Grade Part 33</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -1366,26 +1696,36 @@
         </is>
       </c>
       <c r="E34" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="F34" t="n">
-        <v>172</v>
+        <v>505</v>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SKU-BATCH-034</t>
+          <t>SKU-ERP-0034</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 34</t>
+          <t>Enterprise High-Grade Part 34</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -1394,26 +1734,36 @@
         </is>
       </c>
       <c r="E35" t="n">
-        <v>18</v>
+        <v>48</v>
       </c>
       <c r="F35" t="n">
-        <v>406</v>
+        <v>437</v>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>SKU-BATCH-035</t>
+          <t>SKU-ERP-0035</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 35</t>
+          <t>Enterprise High-Grade Part 35</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -1422,26 +1772,36 @@
         </is>
       </c>
       <c r="E36" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="F36" t="n">
-        <v>328</v>
+        <v>383</v>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SKU-BATCH-036</t>
+          <t>SKU-ERP-0036</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 36</t>
+          <t>Enterprise High-Grade Part 36</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -1450,26 +1810,36 @@
         </is>
       </c>
       <c r="E37" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F37" t="n">
-        <v>275</v>
+        <v>299</v>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SKU-BATCH-037</t>
+          <t>SKU-ERP-0037</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 37</t>
+          <t>Enterprise High-Grade Part 37</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -1478,26 +1848,36 @@
         </is>
       </c>
       <c r="E38" t="n">
-        <v>12</v>
+        <v>37</v>
       </c>
       <c r="F38" t="n">
-        <v>396</v>
+        <v>698</v>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SKU-BATCH-038</t>
+          <t>SKU-ERP-0038</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 38</t>
+          <t>Enterprise High-Grade Part 38</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -1506,26 +1886,36 @@
         </is>
       </c>
       <c r="E39" t="n">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F39" t="n">
-        <v>63</v>
+        <v>86</v>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>SKU-BATCH-039</t>
+          <t>SKU-ERP-0039</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 39</t>
+          <t>Enterprise High-Grade Part 39</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -1534,26 +1924,36 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="F40" t="n">
-        <v>476</v>
+        <v>204</v>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SKU-BATCH-040</t>
+          <t>SKU-ERP-0040</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 40</t>
+          <t>Enterprise High-Grade Part 40</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -1562,26 +1962,36 @@
         </is>
       </c>
       <c r="E41" t="n">
-        <v>29</v>
+        <v>16</v>
       </c>
       <c r="F41" t="n">
-        <v>127</v>
+        <v>556</v>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>SKU-BATCH-041</t>
+          <t>SKU-ERP-0041</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 41</t>
+          <t>Enterprise High-Grade Part 41</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -1590,21 +2000,31 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="F42" t="n">
-        <v>423</v>
+        <v>799</v>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SKU-BATCH-042</t>
+          <t>SKU-ERP-0042</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 42</t>
+          <t>Enterprise High-Grade Part 42</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1618,26 +2038,36 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F43" t="n">
-        <v>59</v>
+        <v>703</v>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>SKU-BATCH-043</t>
+          <t>SKU-ERP-0043</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 43</t>
+          <t>Enterprise High-Grade Part 43</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -1646,21 +2076,31 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>48</v>
+        <v>12</v>
       </c>
       <c r="F44" t="n">
-        <v>451</v>
+        <v>647</v>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SKU-BATCH-044</t>
+          <t>SKU-ERP-0044</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 44</t>
+          <t>Enterprise High-Grade Part 44</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1674,21 +2114,31 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>22</v>
+        <v>44</v>
       </c>
       <c r="F45" t="n">
-        <v>291</v>
+        <v>656</v>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SKU-BATCH-045</t>
+          <t>SKU-ERP-0045</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 45</t>
+          <t>Enterprise High-Grade Part 45</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1702,26 +2152,36 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="F46" t="n">
-        <v>172</v>
+        <v>932</v>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SKU-BATCH-046</t>
+          <t>SKU-ERP-0046</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 46</t>
+          <t>Enterprise High-Grade Part 46</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1730,26 +2190,36 @@
         </is>
       </c>
       <c r="E47" t="n">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F47" t="n">
-        <v>318</v>
+        <v>177</v>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>SKU-BATCH-047</t>
+          <t>SKU-ERP-0047</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 47</t>
+          <t>Enterprise High-Grade Part 47</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1758,21 +2228,31 @@
         </is>
       </c>
       <c r="E48" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="F48" t="n">
-        <v>166</v>
+        <v>499</v>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SKU-BATCH-048</t>
+          <t>SKU-ERP-0048</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 48</t>
+          <t>Enterprise High-Grade Part 48</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -1786,21 +2266,31 @@
         </is>
       </c>
       <c r="E49" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="F49" t="n">
-        <v>430</v>
+        <v>742</v>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>SKU-BATCH-049</t>
+          <t>SKU-ERP-0049</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 49</t>
+          <t>Enterprise High-Grade Part 49</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -1814,26 +2304,36 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>15</v>
+        <v>33</v>
       </c>
       <c r="F50" t="n">
-        <v>127</v>
+        <v>997</v>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>SKU-BATCH-050</t>
+          <t>SKU-ERP-0050</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 50</t>
+          <t>Enterprise High-Grade Part 50</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1842,26 +2342,36 @@
         </is>
       </c>
       <c r="E51" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F51" t="n">
-        <v>465</v>
+        <v>665</v>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SKU-BATCH-051</t>
+          <t>SKU-ERP-0051</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 51</t>
+          <t>Enterprise High-Grade Part 51</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -1870,21 +2380,31 @@
         </is>
       </c>
       <c r="E52" t="n">
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="F52" t="n">
-        <v>125</v>
+        <v>848</v>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SKU-BATCH-052</t>
+          <t>SKU-ERP-0052</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 52</t>
+          <t>Enterprise High-Grade Part 52</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -1898,26 +2418,36 @@
         </is>
       </c>
       <c r="E53" t="n">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="F53" t="n">
-        <v>198</v>
+        <v>230</v>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SKU-BATCH-053</t>
+          <t>SKU-ERP-0053</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 53</t>
+          <t>Enterprise High-Grade Part 53</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -1926,26 +2456,36 @@
         </is>
       </c>
       <c r="E54" t="n">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="F54" t="n">
-        <v>489</v>
+        <v>626</v>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SKU-BATCH-054</t>
+          <t>SKU-ERP-0054</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 54</t>
+          <t>Enterprise High-Grade Part 54</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -1954,21 +2494,31 @@
         </is>
       </c>
       <c r="E55" t="n">
-        <v>14</v>
+        <v>28</v>
       </c>
       <c r="F55" t="n">
-        <v>497</v>
+        <v>442</v>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SKU-BATCH-055</t>
+          <t>SKU-ERP-0055</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 55</t>
+          <t>Enterprise High-Grade Part 55</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -1982,26 +2532,36 @@
         </is>
       </c>
       <c r="E56" t="n">
-        <v>33</v>
+        <v>18</v>
       </c>
       <c r="F56" t="n">
-        <v>420</v>
+        <v>811</v>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SKU-BATCH-056</t>
+          <t>SKU-ERP-0056</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 56</t>
+          <t>Enterprise High-Grade Part 56</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -2010,26 +2570,36 @@
         </is>
       </c>
       <c r="E57" t="n">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="F57" t="n">
-        <v>395</v>
+        <v>517</v>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SKU-BATCH-057</t>
+          <t>SKU-ERP-0057</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 57</t>
+          <t>Enterprise High-Grade Part 57</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -2038,26 +2608,36 @@
         </is>
       </c>
       <c r="E58" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="F58" t="n">
-        <v>442</v>
+        <v>984</v>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SKU-BATCH-058</t>
+          <t>SKU-ERP-0058</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 58</t>
+          <t>Enterprise High-Grade Part 58</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
@@ -2066,26 +2646,36 @@
         </is>
       </c>
       <c r="E59" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="F59" t="n">
-        <v>197</v>
+        <v>792</v>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>SKU-BATCH-059</t>
+          <t>SKU-ERP-0059</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 59</t>
+          <t>Enterprise High-Grade Part 59</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2094,26 +2684,36 @@
         </is>
       </c>
       <c r="E60" t="n">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="F60" t="n">
-        <v>474</v>
+        <v>92</v>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SKU-BATCH-060</t>
+          <t>SKU-ERP-0060</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 60</t>
+          <t>Enterprise High-Grade Part 60</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2122,26 +2722,36 @@
         </is>
       </c>
       <c r="E61" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F61" t="n">
-        <v>273</v>
+        <v>525</v>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>SKU-BATCH-061</t>
+          <t>SKU-ERP-0061</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 61</t>
+          <t>Enterprise High-Grade Part 61</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2150,21 +2760,31 @@
         </is>
       </c>
       <c r="E62" t="n">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="F62" t="n">
-        <v>349</v>
+        <v>497</v>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SKU-BATCH-062</t>
+          <t>SKU-ERP-0062</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 62</t>
+          <t>Enterprise High-Grade Part 62</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2178,26 +2798,36 @@
         </is>
       </c>
       <c r="E63" t="n">
-        <v>36</v>
+        <v>42</v>
       </c>
       <c r="F63" t="n">
-        <v>106</v>
+        <v>127</v>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SKU-BATCH-063</t>
+          <t>SKU-ERP-0063</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 63</t>
+          <t>Enterprise High-Grade Part 63</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
@@ -2206,26 +2836,36 @@
         </is>
       </c>
       <c r="E64" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F64" t="n">
-        <v>152</v>
+        <v>466</v>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SKU-BATCH-064</t>
+          <t>SKU-ERP-0064</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 64</t>
+          <t>Enterprise High-Grade Part 64</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -2234,26 +2874,36 @@
         </is>
       </c>
       <c r="E65" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F65" t="n">
-        <v>197</v>
+        <v>449</v>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SKU-BATCH-065</t>
+          <t>SKU-ERP-0065</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 65</t>
+          <t>Enterprise High-Grade Part 65</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
@@ -2262,26 +2912,36 @@
         </is>
       </c>
       <c r="E66" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="F66" t="n">
-        <v>442</v>
+        <v>986</v>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SKU-BATCH-066</t>
+          <t>SKU-ERP-0066</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 66</t>
+          <t>Enterprise High-Grade Part 66</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -2290,21 +2950,31 @@
         </is>
       </c>
       <c r="E67" t="n">
-        <v>15</v>
+        <v>42</v>
       </c>
       <c r="F67" t="n">
-        <v>130</v>
+        <v>942</v>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SKU-BATCH-067</t>
+          <t>SKU-ERP-0067</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 67</t>
+          <t>Enterprise High-Grade Part 67</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -2318,26 +2988,36 @@
         </is>
       </c>
       <c r="E68" t="n">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="F68" t="n">
-        <v>489</v>
+        <v>99</v>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SKU-BATCH-068</t>
+          <t>SKU-ERP-0068</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 68</t>
+          <t>Enterprise High-Grade Part 68</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -2346,26 +3026,36 @@
         </is>
       </c>
       <c r="E69" t="n">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="F69" t="n">
-        <v>210</v>
+        <v>98</v>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SKU-BATCH-069</t>
+          <t>SKU-ERP-0069</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 69</t>
+          <t>Enterprise High-Grade Part 69</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2374,26 +3064,36 @@
         </is>
       </c>
       <c r="E70" t="n">
-        <v>12</v>
+        <v>42</v>
       </c>
       <c r="F70" t="n">
-        <v>84</v>
+        <v>472</v>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SKU-BATCH-070</t>
+          <t>SKU-ERP-0070</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 70</t>
+          <t>Enterprise High-Grade Part 70</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
@@ -2402,21 +3102,31 @@
         </is>
       </c>
       <c r="E71" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="F71" t="n">
-        <v>159</v>
+        <v>715</v>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SKU-BATCH-071</t>
+          <t>SKU-ERP-0071</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 71</t>
+          <t>Enterprise High-Grade Part 71</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -2430,26 +3140,36 @@
         </is>
       </c>
       <c r="E72" t="n">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="F72" t="n">
-        <v>433</v>
+        <v>641</v>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SKU-BATCH-072</t>
+          <t>SKU-ERP-0072</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 72</t>
+          <t>Enterprise High-Grade Part 72</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2458,26 +3178,36 @@
         </is>
       </c>
       <c r="E73" t="n">
-        <v>50</v>
+        <v>23</v>
       </c>
       <c r="F73" t="n">
-        <v>402</v>
+        <v>585</v>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SKU-BATCH-073</t>
+          <t>SKU-ERP-0073</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 73</t>
+          <t>Enterprise High-Grade Part 73</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -2486,26 +3216,36 @@
         </is>
       </c>
       <c r="E74" t="n">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="F74" t="n">
-        <v>99</v>
+        <v>931</v>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>SKU-BATCH-074</t>
+          <t>SKU-ERP-0074</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 74</t>
+          <t>Enterprise High-Grade Part 74</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -2514,21 +3254,31 @@
         </is>
       </c>
       <c r="E75" t="n">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="F75" t="n">
-        <v>400</v>
+        <v>216</v>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>SKU-BATCH-075</t>
+          <t>SKU-ERP-0075</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 75</t>
+          <t>Enterprise High-Grade Part 75</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -2542,21 +3292,31 @@
         </is>
       </c>
       <c r="E76" t="n">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="F76" t="n">
-        <v>228</v>
+        <v>56</v>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>SKU-BATCH-076</t>
+          <t>SKU-ERP-0076</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 76</t>
+          <t>Enterprise High-Grade Part 76</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -2570,26 +3330,36 @@
         </is>
       </c>
       <c r="E77" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="F77" t="n">
-        <v>305</v>
+        <v>467</v>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>SKU-BATCH-077</t>
+          <t>SKU-ERP-0077</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 77</t>
+          <t>Enterprise High-Grade Part 77</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -2598,26 +3368,36 @@
         </is>
       </c>
       <c r="E78" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F78" t="n">
-        <v>234</v>
+        <v>754</v>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>SKU-BATCH-078</t>
+          <t>SKU-ERP-0078</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 78</t>
+          <t>Enterprise High-Grade Part 78</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -2626,26 +3406,36 @@
         </is>
       </c>
       <c r="E79" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F79" t="n">
-        <v>172</v>
+        <v>374</v>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>SKU-BATCH-079</t>
+          <t>SKU-ERP-0079</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 79</t>
+          <t>Enterprise High-Grade Part 79</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2654,26 +3444,36 @@
         </is>
       </c>
       <c r="E80" t="n">
-        <v>19</v>
+        <v>36</v>
       </c>
       <c r="F80" t="n">
-        <v>466</v>
+        <v>485</v>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>SKU-BATCH-080</t>
+          <t>SKU-ERP-0080</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 80</t>
+          <t>Enterprise High-Grade Part 80</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -2682,26 +3482,36 @@
         </is>
       </c>
       <c r="E81" t="n">
-        <v>48</v>
+        <v>24</v>
       </c>
       <c r="F81" t="n">
-        <v>416</v>
+        <v>445</v>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>SKU-BATCH-081</t>
+          <t>SKU-ERP-0081</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 81</t>
+          <t>Enterprise High-Grade Part 81</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -2710,21 +3520,31 @@
         </is>
       </c>
       <c r="E82" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="F82" t="n">
-        <v>264</v>
+        <v>118</v>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>SKU-BATCH-082</t>
+          <t>SKU-ERP-0082</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 82</t>
+          <t>Enterprise High-Grade Part 82</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -2738,26 +3558,36 @@
         </is>
       </c>
       <c r="E83" t="n">
-        <v>49</v>
+        <v>11</v>
       </c>
       <c r="F83" t="n">
-        <v>319</v>
+        <v>656</v>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>SKU-BATCH-083</t>
+          <t>SKU-ERP-0083</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 83</t>
+          <t>Enterprise High-Grade Part 83</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -2766,26 +3596,36 @@
         </is>
       </c>
       <c r="E84" t="n">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="F84" t="n">
-        <v>458</v>
+        <v>439</v>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>SKU-BATCH-084</t>
+          <t>SKU-ERP-0084</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 84</t>
+          <t>Enterprise High-Grade Part 84</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -2794,26 +3634,36 @@
         </is>
       </c>
       <c r="E85" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="F85" t="n">
-        <v>409</v>
+        <v>337</v>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>SKU-BATCH-085</t>
+          <t>SKU-ERP-0085</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 85</t>
+          <t>Enterprise High-Grade Part 85</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -2822,26 +3672,36 @@
         </is>
       </c>
       <c r="E86" t="n">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="F86" t="n">
-        <v>368</v>
+        <v>290</v>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>SKU-BATCH-086</t>
+          <t>SKU-ERP-0086</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 86</t>
+          <t>Enterprise High-Grade Part 86</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Hardware</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -2850,26 +3710,36 @@
         </is>
       </c>
       <c r="E87" t="n">
-        <v>45</v>
+        <v>17</v>
       </c>
       <c r="F87" t="n">
-        <v>112</v>
+        <v>373</v>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>SKU-BATCH-087</t>
+          <t>SKU-ERP-0087</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 87</t>
+          <t>Enterprise High-Grade Part 87</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -2878,21 +3748,31 @@
         </is>
       </c>
       <c r="E88" t="n">
-        <v>30</v>
+        <v>13</v>
       </c>
       <c r="F88" t="n">
-        <v>185</v>
+        <v>333</v>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>SKU-BATCH-088</t>
+          <t>SKU-ERP-0088</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 88</t>
+          <t>Enterprise High-Grade Part 88</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -2906,26 +3786,36 @@
         </is>
       </c>
       <c r="E89" t="n">
-        <v>47</v>
+        <v>29</v>
       </c>
       <c r="F89" t="n">
-        <v>494</v>
+        <v>453</v>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>SKU-BATCH-089</t>
+          <t>SKU-ERP-0089</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 89</t>
+          <t>Enterprise High-Grade Part 89</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -2934,26 +3824,36 @@
         </is>
       </c>
       <c r="E90" t="n">
-        <v>11</v>
+        <v>43</v>
       </c>
       <c r="F90" t="n">
-        <v>160</v>
+        <v>650</v>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SKU-BATCH-090</t>
+          <t>SKU-ERP-0090</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 90</t>
+          <t>Enterprise High-Grade Part 90</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Electronic</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -2962,26 +3862,36 @@
         </is>
       </c>
       <c r="E91" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="F91" t="n">
-        <v>150</v>
+        <v>859</v>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>SKU-BATCH-091</t>
+          <t>SKU-ERP-0091</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 91</t>
+          <t>Enterprise High-Grade Part 91</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -2990,26 +3900,36 @@
         </is>
       </c>
       <c r="E92" t="n">
-        <v>50</v>
+        <v>12</v>
       </c>
       <c r="F92" t="n">
-        <v>116</v>
+        <v>720</v>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>SKU-BATCH-092</t>
+          <t>SKU-ERP-0092</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 92</t>
+          <t>Enterprise High-Grade Part 92</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -3018,26 +3938,36 @@
         </is>
       </c>
       <c r="E93" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F93" t="n">
-        <v>421</v>
+        <v>766</v>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>SKU-BATCH-093</t>
+          <t>SKU-ERP-0093</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 93</t>
+          <t>Enterprise High-Grade Part 93</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -3046,26 +3976,36 @@
         </is>
       </c>
       <c r="E94" t="n">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="F94" t="n">
-        <v>261</v>
+        <v>594</v>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>SKU-BATCH-094</t>
+          <t>SKU-ERP-0094</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 94</t>
+          <t>Enterprise High-Grade Part 94</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Safety</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
@@ -3074,26 +4014,36 @@
         </is>
       </c>
       <c r="E95" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F95" t="n">
-        <v>87</v>
+        <v>52</v>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>SKU-BATCH-095</t>
+          <t>SKU-ERP-0095</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 95</t>
+          <t>Enterprise High-Grade Part 95</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Fluid</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
@@ -3102,21 +4052,31 @@
         </is>
       </c>
       <c r="E96" t="n">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="F96" t="n">
-        <v>80</v>
+        <v>183</v>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SKU-BATCH-096</t>
+          <t>SKU-ERP-0096</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 96</t>
+          <t>Enterprise High-Grade Part 96</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -3130,26 +4090,36 @@
         </is>
       </c>
       <c r="E97" t="n">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="F97" t="n">
-        <v>320</v>
+        <v>570</v>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SKU-BATCH-097</t>
+          <t>SKU-ERP-0097</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 97</t>
+          <t>Enterprise High-Grade Part 97</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Hardware</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -3158,26 +4128,36 @@
         </is>
       </c>
       <c r="E98" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="F98" t="n">
-        <v>241</v>
+        <v>432</v>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SKU-BATCH-098</t>
+          <t>SKU-ERP-0098</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 98</t>
+          <t>Enterprise High-Grade Part 98</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Safety</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
@@ -3186,21 +4166,31 @@
         </is>
       </c>
       <c r="E99" t="n">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="F99" t="n">
-        <v>53</v>
+        <v>58</v>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SKU-BATCH-099</t>
+          <t>SKU-ERP-0099</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 99</t>
+          <t>Enterprise High-Grade Part 99</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -3214,26 +4204,36 @@
         </is>
       </c>
       <c r="E100" t="n">
-        <v>42</v>
+        <v>26</v>
       </c>
       <c r="F100" t="n">
-        <v>460</v>
+        <v>206</v>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SKU-BATCH-100</t>
+          <t>SKU-ERP-0100</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Enterprise Component Pro 100</t>
+          <t>Enterprise High-Grade Part 100</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Fluid</t>
+          <t>Electronic</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
@@ -3242,10 +4242,20 @@
         </is>
       </c>
       <c r="E101" t="n">
-        <v>37</v>
+        <v>42</v>
       </c>
       <c r="F101" t="n">
-        <v>195</v>
+        <v>324</v>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>2025-01-01</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>